<commit_message>
Add complete bilingual abstract column to coarse reading
</commit_message>
<xml_diff>
--- a/assets/coarse-reading-template.xlsx
+++ b/assets/coarse-reading-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文粗读" sheetId="1" r:id="R8d7aeb64054e41b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文粗读" sheetId="1" r:id="Rbafa60a843f44e02"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -45,6 +45,11 @@
     </x:font>
     <x:font>
       <x:sz val="14"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="等线"/>
+    </x:font>
+    <x:font>
+      <x:sz val="12"/>
       <x:color rgb="FF222222"/>
       <x:name val="等线"/>
     </x:font>
@@ -106,7 +111,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="34">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -179,6 +184,9 @@
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -187,17 +195,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PaperReadingTable" displayName="PaperReadingTable" ref="A1:H2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H2"/>
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PaperReadingTable" displayName="PaperReadingTable" ref="A1:I2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:I2"/>
+  <x:tableColumns count="9">
     <x:tableColumn id="1" name="论文题目"/>
     <x:tableColumn id="2" name="作者及机构"/>
-    <x:tableColumn id="3" name="关键词"/>
-    <x:tableColumn id="4" name="针对的问题"/>
-    <x:tableColumn id="5" name="解决的方法"/>
-    <x:tableColumn id="6" name="创新以及借鉴地方"/>
-    <x:tableColumn id="7" name="代码位置"/>
-    <x:tableColumn id="8" name="批判地方"/>
+    <x:tableColumn id="3" name="摘要"/>
+    <x:tableColumn id="4" name="关键词"/>
+    <x:tableColumn id="5" name="针对的问题"/>
+    <x:tableColumn id="6" name="解决的方法"/>
+    <x:tableColumn id="7" name="创新以及借鉴地方"/>
+    <x:tableColumn id="8" name="代码位置"/>
+    <x:tableColumn id="9" name="批判地方"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -400,12 +409,13 @@
   <x:cols>
     <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="70" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="41" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="100" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="70" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="41" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="60" customHeight="1">
@@ -415,39 +425,43 @@
       <x:c r="B1" s="8" t="str">
         <x:v>作者及机构</x:v>
       </x:c>
-      <x:c r="C1" s="12" t="str">
+      <x:c r="C1" s="8" t="str">
+        <x:v>摘要</x:v>
+      </x:c>
+      <x:c r="D1" s="12" t="str">
         <x:v>关键词</x:v>
       </x:c>
-      <x:c r="D1" s="8" t="str">
+      <x:c r="E1" s="8" t="str">
         <x:v>针对的问题</x:v>
       </x:c>
-      <x:c r="E1" s="16" t="str">
+      <x:c r="F1" s="16" t="str">
         <x:v>解决的方法</x:v>
       </x:c>
-      <x:c r="F1" s="8" t="str">
+      <x:c r="G1" s="8" t="str">
         <x:v>创新以及借鉴地方</x:v>
       </x:c>
-      <x:c r="G1" s="19" t="str">
+      <x:c r="H1" s="19" t="str">
         <x:v>代码位置</x:v>
       </x:c>
-      <x:c r="H1" s="8" t="str">
+      <x:c r="I1" s="8" t="str">
         <x:v>批判地方</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="31" t="str"/>
       <x:c r="B2" s="32" t="str"/>
-      <x:c r="C2" s="32" t="str"/>
+      <x:c r="C2" s="34" t="str"/>
       <x:c r="D2" s="32" t="str"/>
       <x:c r="E2" s="32" t="str"/>
       <x:c r="F2" s="32" t="str"/>
       <x:c r="G2" s="32" t="str"/>
-      <x:c r="H2" s="33" t="str"/>
+      <x:c r="H2" s="32" t="str"/>
+      <x:c r="I2" s="33" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5237cee9a9674fca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4792c13f784d4c46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>